<commit_message>
Melhorando lógica do Web Scrapping (erro 403)
</commit_message>
<xml_diff>
--- a/planilhas_geradas/planilha_casas.xlsx
+++ b/planilhas_geradas/planilha_casas.xlsx
@@ -26,18 +26,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,14 +54,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4B4B4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -422,35 +448,35 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Índice</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Link do anúncio</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Endereço</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Telefone da imobiliária</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Telefone do vendedor</t>
         </is>

</xml_diff>

<commit_message>
FINALIZADO - VERSAO 1
</commit_message>
<xml_diff>
--- a/planilhas_geradas/planilha_casas.xlsx
+++ b/planilhas_geradas/planilha_casas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Casas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +31,24 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00404040"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+        <bgColor rgb="00F5F7FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,13 +94,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,14 +497,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="54" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -473,16 +526,806 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Tamanho (m²)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>Telefone da imobiliária</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Telefone do vendedor</t>
         </is>
       </c>
     </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-60m2-venda-RS490000-id-2885560930/</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Itaquera para venda com Cozinha, 60 m² por R$ 490.000,00. Entre em contato com GRUPO URBAN IMÓVEIS!</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>2885560930</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS555000-id-2846899225/</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 100 m² por R$ 555.000,00. Entre em contato com Coroa Real Imóveis!</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>2846899225</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-87m2-venda-RS350000-id-2748510414/</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Itaquera para venda com  , 87 m² por R$ 350.000,00. Entre em contato com Catita Imóveis!</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>2748510414</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS540000-id-2803432496/</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Itaquera para venda com Cozinha, 120 m² por R$ 540.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>2803432496</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS426000-id-2652589154/</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 100 m² por R$ 426.000,00. Entre em contato com Catita Imóveis!</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>2652589154</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-114m2-venda-RS1200000-id-2879443210/</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Piscina, 114 m² por R$ 1.200.000,00. Entre em contato com Foxter SP!</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>2879443210</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-160m2-venda-RS980100-id-2885033261/</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Mobiliado, 160 m² por R$ 980.100,00. Entre em contato com L.G.K.G. - NEGOCIOS IMOBILIARIOS!</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>2885033261</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-165m2-venda-RS555000-id-2859937056/</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 165 m² por R$ 555.000,00. Entre em contato com Lello Vendas!</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>2859937056</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-183m2-venda-RS1280000-id-2733176226/</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 183 m² por R$ 1.280.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>2733176226</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-187m2-venda-RS750000-id-2881941392/</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 187 m² por R$ 750.000,00. Entre em contato com Crédito Real | Leroi!</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>2881941392</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-200m2-venda-RS460000-id-2885954780/</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Itaquera para venda com Mobiliado, 200 m² por R$ 460.000,00. Entre em contato com benedito aparecido finhana!</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>2885954780</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-itaquera-zona-leste-sao-paulo-com-garagem-160m2-venda-RS750000-id-2886015986/</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Itaquera para venda com :amenity, 160 m² por R$ 750.000,00. Entre em contato com Re/Max Nova Esperança!</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>2886015986</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-290m2-venda-RS841500-id-2885035019/</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Sacada, 290 m² por R$ 841.500,00. Entre em contato com L.G.K.G. - NEGOCIOS IMOBILIARIOS!</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>290</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>2885035019</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-480m2-venda-RS1060000-id-2829836527/</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Casas na Zona Leste em Cidade Patriarca para venda com Área de serviço, 480 m² por R$ 1.060.000,00. Entre em contato com Foxter SP!</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>2829836527</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-105m2-venda-RS560000-id-2737992892/</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 105 m² por R$ 560.000,00. Entre em contato com Thiago Imóveis!</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>2737992892</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-110m2-venda-RS680000-id-2856436117/</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 110 m² por R$ 680.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>2856436117</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS680000-id-2846900139/</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 120 m² por R$ 680.000,00. Entre em contato com Coroa Real Imóveis!</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2846900139</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-130m2-venda-RS600000-id-2841868511/</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 130 m² por R$ 600.000,00. Entre em contato com Special Imóveis - Tatuapé!</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>2841868511</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-146m2-venda-RS560000-id-2860951156/</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 146 m² por R$ 560.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>2860951156</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS550000-id-2599470254/</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 150 m² por R$ 550.000,00. Entre em contato com Marengo Imoveis Ltda.!</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>2599470254</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-71m2-venda-RS480000-id-2884956208/</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Sacada, 71 m² por R$ 480.000,00. Entre em contato com Df Casa Imoveis!</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>2884956208</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-93m2-venda-RS550000-id-2878779118/</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Interfone, 93 m² por R$ 550.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>2878779118</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-122m2-venda-RS500000-id-2871022821/</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com Churrasqueira, 122 m² por R$ 500.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>2871022821</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-62m2-venda-RS420000-id-2811541725/</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com  , 62 m² por R$ 420.000,00. Entre em contato com Catita Imóveis!</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>2811541725</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS350000-id-2881477776/</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com  , 65 m² por R$ 350.000,00. Entre em contato com Df Casa Imoveis!</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>2881477776</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-81m2-venda-RS420000-id-2718762034/</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com  , 81 m² por R$ 420.000,00. Entre em contato com Df Casa Imoveis!</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>2718762034</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-82m2-venda-RS400000-id-2718758947/</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com  , 82 m² por R$ 400.000,00. Entre em contato com Df Casa Imoveis!</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>2718758947</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-100m2-venda-RS550000-id-2871872166/</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Itaquera para venda com Churrasqueira, 100 m² por R$ 550.000,00. Entre em contato com Yamakawa Imóveis!</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>2871872166</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30" ht="38" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS700000-id-2818021087/</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Mobiliado, 100 m² por R$ 700.000,00. Entre em contato com Parceiro Imóveis!</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>2818021087</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustando coluna de enderecos
</commit_message>
<xml_diff>
--- a/planilhas_geradas/planilha_casas.xlsx
+++ b/planilhas_geradas/planilha_casas.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -546,22 +546,22 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-60m2-venda-RS490000-id-2885560930/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-70m2-venda-RS480000-id-2874947265/</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Itaquera para venda com Cozinha, 60 m² por R$ 490.000,00. Entre em contato com GRUPO URBAN IMÓVEIS!</t>
+          <t>Avenida Engenheiro Soares de Camargo, 191 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>70</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>2885560930</t>
+          <t>2874947265</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr"/>
@@ -572,22 +572,22 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS555000-id-2846899225/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-280m2-venda-RS750000-id-2832708315/</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 100 m² por R$ 555.000,00. Entre em contato com Coroa Real Imóveis!</t>
+          <t>Rua Pedro Morcilla Filho, 252 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>280</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>2846899225</t>
+          <t>2832708315</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr"/>
@@ -598,22 +598,22 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-87m2-venda-RS350000-id-2748510414/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-293m2-venda-RS670000-id-2863398959/</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Itaquera para venda com  , 87 m² por R$ 350.000,00. Entre em contato com Catita Imóveis!</t>
+          <t>Rua Baixada Santista, 839 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>293</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>2748510414</t>
+          <t>2863398959</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
@@ -624,22 +624,22 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS540000-id-2803432496/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-168m2-venda-RS940500-id-2885043630/</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Itaquera para venda com Cozinha, 120 m² por R$ 540.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>Rua Padre Salvador Machado, 186 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>168</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>2803432496</t>
+          <t>2885043630</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr"/>
@@ -650,22 +650,22 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS426000-id-2652589154/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-150m2-venda-RS950000-id-2881943374/</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 100 m² por R$ 426.000,00. Entre em contato com Catita Imóveis!</t>
+          <t>Rua Freguesia de Poiares, 26 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>150</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>2652589154</t>
+          <t>2881943374</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr"/>
@@ -676,22 +676,22 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-114m2-venda-RS1200000-id-2879443210/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-itaquera-zona-leste-sao-paulo-com-garagem-160m2-venda-RS750000-id-2886015986/</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Piscina, 114 m² por R$ 1.200.000,00. Entre em contato com Foxter SP!</t>
+          <t>Avenida Doutor Francisco Munhoz Filho, 76 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>160</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>2879443210</t>
+          <t>2886015986</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr"/>
@@ -702,22 +702,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-160m2-venda-RS980100-id-2885033261/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-7-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-270m2-venda-RS979000-id-2885561121/</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Mobiliado, 160 m² por R$ 980.100,00. Entre em contato com L.G.K.G. - NEGOCIOS IMOBILIARIOS!</t>
+          <t>Rua Videira, 43 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>2885033261</t>
+          <t>2885561121</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr"/>
@@ -728,22 +728,22 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-165m2-venda-RS555000-id-2859937056/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-de-condominio-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-84m2-venda-RS532000-id-2694787983/</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 165 m² por R$ 555.000,00. Entre em contato com Lello Vendas!</t>
+          <t>Rua Antônio Soares Lara, 72 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>84</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>2859937056</t>
+          <t>2694787983</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr"/>
@@ -754,22 +754,22 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-183m2-venda-RS1280000-id-2733176226/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-86m2-venda-RS670000-id-2857364659/</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 183 m² por R$ 1.280.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>Rua Sebastião Daniel de Sousa, 900 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>86</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2733176226</t>
+          <t>2857364659</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
@@ -780,22 +780,22 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-187m2-venda-RS750000-id-2881941392/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-95m2-venda-RS598000-id-2830783124/</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 187 m² por R$ 750.000,00. Entre em contato com Crédito Real | Leroi!</t>
+          <t>Rua Palmeiras das Missões, 35 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>95</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>2881941392</t>
+          <t>2830783124</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr"/>
@@ -806,22 +806,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-200m2-venda-RS460000-id-2885954780/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-60m2-venda-RS380000-id-2874456885/</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Itaquera para venda com Mobiliado, 200 m² por R$ 460.000,00. Entre em contato com benedito aparecido finhana!</t>
+          <t>Rua Barra de Guabiraba, 30 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>2885954780</t>
+          <t>2874456885</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr"/>
@@ -832,22 +832,22 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-itaquera-zona-leste-sao-paulo-com-garagem-160m2-venda-RS750000-id-2886015986/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS373000-id-2875587077/</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Itaquera para venda com :amenity, 160 m² por R$ 750.000,00. Entre em contato com Re/Max Nova Esperança!</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>2886015986</t>
+          <t>2875587077</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr"/>
@@ -858,22 +858,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-290m2-venda-RS841500-id-2885035019/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-70m2-venda-RS440000-id-2834053172/</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Sacada, 290 m² por R$ 841.500,00. Entre em contato com L.G.K.G. - NEGOCIOS IMOBILIARIOS!</t>
+          <t>Rua Barra de Guabiraba, 84 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>70</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>2885035019</t>
+          <t>2834053172</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
@@ -884,22 +884,22 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-480m2-venda-RS1060000-id-2829836527/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS380000-id-2823005150/</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Casas na Zona Leste em Cidade Patriarca para venda com Área de serviço, 480 m² por R$ 1.060.000,00. Entre em contato com Foxter SP!</t>
+          <t>Rua Brígida de Vasconcelos, 47 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>2829836527</t>
+          <t>2823005150</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr"/>
@@ -910,22 +910,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-105m2-venda-RS560000-id-2737992892/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS480000-id-2882746406/</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 105 m² por R$ 560.000,00. Entre em contato com Thiago Imóveis!</t>
+          <t>Rua Senador Georgino Avelino, 957 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>2737992892</t>
+          <t>2882746406</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
@@ -936,22 +936,22 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-110m2-venda-RS680000-id-2856436117/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-250m2-venda-RS425000-id-2863348056/</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 110 m² por R$ 680.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>Rua Lagoa Tai Grande, 1288 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>250</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>2856436117</t>
+          <t>2863348056</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr"/>
@@ -962,22 +962,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS680000-id-2846900139/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS400000-id-2872565830/</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 120 m² por R$ 680.000,00. Entre em contato com Coroa Real Imóveis!</t>
+          <t>Rua Harry Dannenberg, 793 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>2846900139</t>
+          <t>2872565830</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
@@ -988,22 +988,22 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-130m2-venda-RS600000-id-2841868511/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS375000-id-2876257517/</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Churrasqueira, 130 m² por R$ 600.000,00. Entre em contato com Special Imóveis - Tatuapé!</t>
+          <t>Rua Catarina Lopes, 237 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>2841868511</t>
+          <t>2876257517</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr"/>
@@ -1014,22 +1014,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-146m2-venda-RS560000-id-2860951156/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-105m2-venda-RS430000-id-2846899223/</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 146 m² por R$ 560.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>105</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>2860951156</t>
+          <t>2846899223</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
@@ -1040,22 +1040,22 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS550000-id-2599470254/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS790000-id-2813436263/</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com  , 150 m² por R$ 550.000,00. Entre em contato com Marengo Imoveis Ltda.!</t>
+          <t>Rua Colatina, 383 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>2599470254</t>
+          <t>2813436263</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr"/>
@@ -1066,22 +1066,22 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-71m2-venda-RS480000-id-2884956208/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-139m2-venda-RS859000-id-2886562580/</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Sacada, 71 m² por R$ 480.000,00. Entre em contato com Df Casa Imoveis!</t>
+          <t>Rua Clevelândia, 280 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>139</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>2884956208</t>
+          <t>2886562580</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
@@ -1092,22 +1092,22 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-93m2-venda-RS550000-id-2878779118/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS700000-id-2751725095/</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Interfone, 93 m² por R$ 550.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>Rua Vitória da Conquista, 188 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>150</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>2878779118</t>
+          <t>2751725095</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr"/>
@@ -1118,22 +1118,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-122m2-venda-RS500000-id-2871022821/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS830000-id-2813437748/</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com Churrasqueira, 122 m² por R$ 500.000,00. Entre em contato com Yamakawa Imóveis!</t>
+          <t>Rua Castanhal, 108 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>150</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>2871022821</t>
+          <t>2813437748</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
@@ -1144,22 +1144,22 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-62m2-venda-RS420000-id-2811541725/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-170m2-venda-RS890000-id-2846896565/</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com  , 62 m² por R$ 420.000,00. Entre em contato com Catita Imóveis!</t>
+          <t>Rua Mazagão, 63 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>170</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>2811541725</t>
+          <t>2846896565</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr"/>
@@ -1170,129 +1170,25 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS350000-id-2881477776/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-280m2-venda-RS960000-id-2818713326/</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com  , 65 m² por R$ 350.000,00. Entre em contato com Df Casa Imoveis!</t>
+          <t>Rua Pedro Morcilla Filho, 230 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>280</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>2881477776</t>
+          <t>2818713326</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-81m2-venda-RS420000-id-2718762034/</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com  , 81 m² por R$ 420.000,00. Entre em contato com Df Casa Imoveis!</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>2718762034</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr"/>
-    </row>
-    <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-82m2-venda-RS400000-id-2718758947/</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com  , 82 m² por R$ 400.000,00. Entre em contato com Df Casa Imoveis!</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>2718758947</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
-    </row>
-    <row r="29" ht="38" customHeight="1">
-      <c r="A29" s="8" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-100m2-venda-RS550000-id-2871872166/</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Sobrados na Zona Leste em Itaquera para venda com Churrasqueira, 100 m² por R$ 550.000,00. Entre em contato com Yamakawa Imóveis!</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>2871872166</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr"/>
-    </row>
-    <row r="30" ht="38" customHeight="1">
-      <c r="A30" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS700000-id-2818021087/</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Sobrados na Zona Leste em Cidade Patriarca para venda com Mobiliado, 100 m² por R$ 700.000,00. Entre em contato com Parceiro Imóveis!</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>2818021087</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1321,10 +1217,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remover Netlify e simplificar instruções do site público no README.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/planilhas_geradas/planilha_casas.xlsx
+++ b/planilhas_geradas/planilha_casas.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -546,22 +546,22 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-70m2-venda-RS480000-id-2874947265/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS599900-id-2746782607/</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Avenida Engenheiro Soares de Camargo, 191 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Cangambá, 120 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>2874947265</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr"/>
@@ -572,22 +572,22 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-280m2-venda-RS750000-id-2832708315/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-87m2-venda-RS350000-id-2748510414/</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Rua Pedro Morcilla Filho, 252 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Acotipa, 209 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>87</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>2832708315</t>
+          <t>(11) 2741-5050</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr"/>
@@ -598,22 +598,22 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-293m2-venda-RS670000-id-2863398959/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS540000-id-2803432496/</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Rua Baixada Santista, 839 - Itaquera, São Paulo - SP</t>
+          <t>Rua Jerônimo de Barros, 232 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>293</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>2863398959</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
@@ -624,22 +624,22 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-168m2-venda-RS940500-id-2885043630/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS426000-id-2652589154/</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Rua Padre Salvador Machado, 186 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Professor Athanassof, 153 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>2885043630</t>
+          <t>(11) 2741-5050</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr"/>
@@ -650,25 +650,29 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-150m2-venda-RS950000-id-2881943374/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-102m2-venda-RS690000-id-2819600217/</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Rua Freguesia de Poiares, 26 - Itaquera, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>102</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>2881943374</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr"/>
+          <t>(11) 96593-5749</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2682-2320</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -676,22 +680,22 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-itaquera-zona-leste-sao-paulo-com-garagem-160m2-venda-RS750000-id-2886015986/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-142m2-venda-RS895000-id-2867240583/</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Avenida Doutor Francisco Munhoz Filho, 76 - Itaquera, São Paulo - SP</t>
+          <t>Avenida Ajarani, 231 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>142</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>2886015986</t>
+          <t>(11) 5071-2679</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr"/>
@@ -702,25 +706,29 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-7-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-270m2-venda-RS979000-id-2885561121/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-90m2-venda-RS650000-id-2543425622/</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Rua Videira, 43 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Xapuri, 56 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>2885561121</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr"/>
+          <t>(11) 96737-5059</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2692-9272</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="8" t="n">
@@ -728,22 +736,22 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-de-condominio-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-84m2-venda-RS532000-id-2694787983/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-200m2-venda-RS500000-id-2887847487/</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Rua Antônio Soares Lara, 72 - Itaquera, São Paulo - SP</t>
+          <t>Rua Doutor Aureliano Barreiros, 606 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>2694787983</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr"/>
@@ -754,25 +762,29 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-86m2-venda-RS670000-id-2857364659/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-250m2-venda-RS675000-id-2848679032/</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Rua Sebastião Daniel de Sousa, 900 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Piraquara, 115 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>250</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2857364659</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr"/>
+          <t>(11) 98885-8836</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>(98) 2421-5021</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="8" t="n">
@@ -780,22 +792,22 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-95m2-venda-RS598000-id-2830783124/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-210m2-venda-RS830000-id-2878358673/</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Rua Palmeiras das Missões, 35 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Pedro Franco Quaresma, 296 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>210</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>2830783124</t>
+          <t>(11) 91495-8731</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr"/>
@@ -806,22 +818,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-60m2-venda-RS380000-id-2874456885/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-de-condominio-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-223m2-venda-RS660000-id-2876036217/</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Rua Barra de Guabiraba, 30 - Itaquera, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>223</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>2874456885</t>
+          <t>(11) 93061-0014</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr"/>
@@ -832,22 +844,22 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS373000-id-2875587077/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-71m2-venda-RS480000-id-2884956208/</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Avenida Engenheiro Soares de Camargo, 262 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>71</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>2875587077</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr"/>
@@ -858,22 +870,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-70m2-venda-RS440000-id-2834053172/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-95m2-venda-RS600000-id-2866982769/</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Rua Barra de Guabiraba, 84 - Itaquera, São Paulo - SP</t>
+          <t>Rua Palmeiras das Missões, 89 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>2834053172</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
@@ -884,22 +896,22 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS380000-id-2823005150/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-81m2-venda-RS420000-id-2718762034/</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Rua Brígida de Vasconcelos, 47 - Itaquera, São Paulo - SP</t>
+          <t>Rua Brígida de Vasconcelos, 163 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>2823005150</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr"/>
@@ -910,22 +922,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS480000-id-2882746406/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-90m2-venda-RS449000-id-2834122819/</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Rua Senador Georgino Avelino, 957 - Itaquera, São Paulo - SP</t>
+          <t>Rua Abelardo Luz, 10 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>2882746406</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
@@ -936,22 +948,22 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-250m2-venda-RS425000-id-2863348056/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-96m2-venda-RS550000-id-2882873079/</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Rua Lagoa Tai Grande, 1288 - Itaquera, São Paulo - SP</t>
+          <t>Rua Barra de Guabiraba, 546 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>2863348056</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr"/>
@@ -962,22 +974,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS400000-id-2872565830/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-267m2-venda-RS599000-id-2746782993/</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Rua Harry Dannenberg, 793 - Itaquera, São Paulo - SP</t>
+          <t>Rua Alfredo Costa, 179 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>267</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>2872565830</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
@@ -988,22 +1000,22 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-80m2-venda-RS375000-id-2876257517/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-63m2-venda-RS450000-id-2871318802/</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Rua Catarina Lopes, 237 - Itaquera, São Paulo - SP</t>
+          <t>Rua da Lagoa Feia, 290 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>63</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>2876257517</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr"/>
@@ -1014,22 +1026,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-105m2-venda-RS430000-id-2846899223/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS299000-id-2880790973/</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Jaguaruna, 210 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>2846899223</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
@@ -1040,12 +1052,12 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS790000-id-2813436263/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS745000-id-2567569232/</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Rua Colatina, 383 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Caicó, 442 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -1055,7 +1067,7 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>2813436263</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr"/>
@@ -1066,25 +1078,29 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-139m2-venda-RS859000-id-2886562580/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS780000-id-2796931955/</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Rua Clevelândia, 280 - Cidade Patriarca, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>2886562580</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr"/>
+          <t>(11) 98635-6646</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>(11) 3772-6265</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="38" customHeight="1">
       <c r="A23" s="8" t="n">
@@ -1092,25 +1108,29 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS700000-id-2751725095/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS795000-id-2774672641/</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Rua Vitória da Conquista, 188 - Cidade Patriarca, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>2751725095</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr"/>
+          <t>(11) 94846-6244</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>(11) 4172-1313</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="38" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -1118,25 +1138,29 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-150m2-venda-RS830000-id-2813437748/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-142m2-venda-RS799000-id-2846900138/</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Rua Castanhal, 108 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Vitória da Conquista, 174 A - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>142</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>2813437748</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
+          <t>(11) 99110-4782</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2744-0100</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="38" customHeight="1">
       <c r="A25" s="8" t="n">
@@ -1144,22 +1168,22 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-170m2-venda-RS890000-id-2846896565/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-160m2-venda-RS1100000-id-2883154123/</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Rua Mazagão, 63 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Marcos Grotti Vidal, 232 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>160</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>2846896565</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr"/>
@@ -1170,25 +1194,171 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-280m2-venda-RS960000-id-2818713326/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-169m2-venda-RS795000-id-2567773185/</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Rua Pedro Morcilla Filho, 230 - Cidade Patriarca, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>169</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>2818713326</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr"/>
+          <t>(11) 96593-5749</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2682-2320</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-190m2-venda-RS890000-id-2869660708/</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Rua Mazagão, 65 - Cidade Patriarca, São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>(11) 2155-8801</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-226m2-venda-RS790000-id-2795163419/</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Rua Marialva, 294 - Cidade Patriarca, São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2385-7633</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-227m2-venda-RS641000-id-2833843713/</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Rua Mazagão, 322 - Cidade Patriarca, São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>(11) 97395-3363</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>(11) 3565-3530</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-263m2-venda-RS990000-id-2804358420/</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>CEP 08079-354</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>(11) 94084-8316</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2958-8884</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="38" customHeight="1">
+      <c r="A31" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-287m2-venda-RS1150000-id-2840293965/</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>CEP 08079-354</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>287</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>(11) 96272-6666</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>(11) 2287-6666</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1217,6 +1387,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refinando filtro de regioes
</commit_message>
<xml_diff>
--- a/planilhas_geradas/planilha_casas.xlsx
+++ b/planilhas_geradas/planilha_casas.xlsx
@@ -546,25 +546,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS599900-id-2746782607/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-145m2-venda-RS580000-id-2843954767/</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Rua Cangambá, 120 - Itaquera, São Paulo - SP</t>
+          <t>Rua Sebastião Daniel de Sousa, 1 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>145</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>(11) 2155-8800</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr"/>
+          <t>(11) 92202-3771</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2672-1212</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="8" t="n">
@@ -572,22 +576,22 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-87m2-venda-RS350000-id-2748510414/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-50m2-venda-RS460000-id-2850304035/</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Rua Acotipa, 209 - Itaquera, São Paulo - SP</t>
+          <t>Rua Dom Joaquim de Oliveira, 316 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>(11) 2741-5050</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr"/>
@@ -598,25 +602,29 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS540000-id-2803432496/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-86m2-venda-RS580000-id-2847071966/</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Rua Jerônimo de Barros, 232 - Itaquera, São Paulo - SP</t>
+          <t>Rua Quintiliano Moreira César, 125 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>86</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>(11) 2155-8800</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr"/>
+          <t>(11) 96593-5749</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2682-2320</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="8" t="n">
@@ -624,22 +632,22 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-100m2-venda-RS426000-id-2652589154/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-108m2-venda-RS460000-id-2888366373/</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Rua Professor Athanassof, 153 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Professor Brito Machado, 135 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>108</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>(11) 2741-5050</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr"/>
@@ -650,29 +658,25 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-102m2-venda-RS690000-id-2819600217/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-120m2-venda-RS540000-id-2803432496/</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Jerônimo de Barros, 232 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>120</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>(11) 96593-5749</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>(11) 2682-2320</t>
-        </is>
-      </c>
+          <t>(11) 2155-8800</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -680,22 +684,22 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-142m2-venda-RS895000-id-2867240583/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-144m2-venda-RS570000-id-2881940714/</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Avenida Ajarani, 231 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Roque Palmieri, 385 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>144</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>(11) 5071-2679</t>
+          <t>(11) 91495-8731</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr"/>
@@ -706,27 +710,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-90m2-venda-RS650000-id-2543425622/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-110m2-venda-RS658990-id-2881942791/</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Rua Xapuri, 56 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Antônio Sampaio Ferraz, 109 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>110</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>(11) 96737-5059</t>
+          <t>(11) 91495-8731</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>(11) 2692-9272</t>
+          <t>(63) 4274-2346</t>
         </is>
       </c>
     </row>
@@ -736,22 +740,22 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-200m2-venda-RS500000-id-2887847487/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-118m2-venda-RS410000-id-2788477818/</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Rua Doutor Aureliano Barreiros, 606 - Itaquera, São Paulo - SP</t>
+          <t>Rua Jatiba, 131 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>118</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>(11) 3571-6696</t>
+          <t>(11) 2741-5050</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr"/>
@@ -762,27 +766,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-itaquera-zona-leste-sao-paulo-com-garagem-250m2-venda-RS675000-id-2848679032/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-4-quartos-itaquera-zona-leste-sao-paulo-com-garagem-160m2-venda-RS750000-id-2880008470/</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Rua Piraquara, 115 - Itaquera, São Paulo - SP</t>
+          <t>Rua Marcelino da Silva, 76 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>160</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>(11) 98885-8836</t>
+          <t>(11) 91146-5011</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>(98) 2421-5021</t>
+          <t>(93) 4496-9951</t>
         </is>
       </c>
     </row>
@@ -792,22 +796,22 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/casa-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-210m2-venda-RS830000-id-2878358673/</t>
+          <t>https://www.vivareal.com.br/imovel/casa-5-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-300m2-venda-RS1060000-id-2813112883/</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Rua Pedro Franco Quaresma, 296 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Mateo Martins Cebantos, 264 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>300</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>(11) 91495-8731</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr"/>
@@ -870,22 +874,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-95m2-venda-RS600000-id-2866982769/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-80m2-venda-RS455000-id-2873714382/</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Rua Palmeiras das Missões, 89 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Avenida Engenheiro Soares de Camargo, 191 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>(11) 3571-6696</t>
+          <t>(11) 2155-8801</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
@@ -896,22 +900,22 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-81m2-venda-RS420000-id-2718762034/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-93m2-venda-RS550000-id-2878779118/</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Rua Brígida de Vasconcelos, 163 - Itaquera, São Paulo - SP</t>
+          <t>Avenida Antônio Estevão de Carvalho, 3444 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>93</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>(11) 3571-6696</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr"/>
@@ -922,22 +926,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-90m2-venda-RS449000-id-2834122819/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-95m2-venda-RS600000-id-2866982769/</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Rua Abelardo Luz, 10 - Itaquera, São Paulo - SP</t>
+          <t>Rua Palmeiras das Missões, 89 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>95</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>(11) 2155-8800</t>
+          <t>(11) 3571-6696</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
@@ -948,22 +952,22 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-96m2-venda-RS550000-id-2882873079/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-62m2-venda-RS420000-id-2811541725/</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Rua Barra de Guabiraba, 546 - Itaquera, São Paulo - SP</t>
+          <t>Rua Lagoa Tai Grande, 1239 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>62</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>(11) 3571-6696</t>
+          <t>(11) 2741-5050</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr"/>
@@ -974,25 +978,29 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-267m2-venda-RS599000-id-2746782993/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-90m2-venda-RS500000-id-2776558153/</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Rua Alfredo Costa, 179 - Itaquera, São Paulo - SP</t>
+          <t>CEP 08079-354</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>267</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>(11) 2155-8800</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr"/>
+          <t>(11) 96593-5749</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2682-2320</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="8" t="n">
@@ -1026,22 +1034,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-65m2-venda-RS299000-id-2880790973/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-2-quartos-itaquera-zona-leste-sao-paulo-com-garagem-83m2-venda-RS530000-id-2865148287/</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Rua Jaguaruna, 210 - Itaquera, São Paulo - SP</t>
+          <t>Rua Rio Fortuna, 59 - Itaquera, São Paulo - SP</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>(11) 3571-6696</t>
+          <t>(11) 2155-8800</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
@@ -1052,17 +1060,17 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS745000-id-2567569232/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-115m2-venda-RS850000-id-2876956474/</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Rua Caicó, 442 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Mantenópolis, 86 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>115</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -1078,27 +1086,27 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS780000-id-2796931955/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-127m2-venda-RS750000-id-2655792659/</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Xique-Xique, 447 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>127</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>(11) 98635-6646</t>
+          <t>(11) 96593-5749</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>(11) 3772-6265</t>
+          <t>(11) 2682-2320</t>
         </is>
       </c>
     </row>
@@ -1108,29 +1116,25 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-120m2-venda-RS795000-id-2774672641/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-130m2-venda-RS626850-id-2875022505/</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Campo Maior, 98 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>130</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>(11) 94846-6244</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>(11) 4172-1313</t>
-        </is>
-      </c>
+          <t>(11) 4228-1111</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr"/>
     </row>
     <row r="24" ht="38" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -1138,29 +1142,25 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-142m2-venda-RS799000-id-2846900138/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-130m2-venda-RS850000-id-2869837301/</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Rua Vitória da Conquista, 174 A - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Araruama, 158 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>130</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>(11) 99110-4782</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>(11) 2744-0100</t>
-        </is>
-      </c>
+          <t>(11) 2155-8800</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="38" customHeight="1">
       <c r="A25" s="8" t="n">
@@ -1168,25 +1168,29 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-160m2-venda-RS1100000-id-2883154123/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-133m2-venda-RS840000-id-2870252227/</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Rua Marcos Grotti Vidal, 232 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Avenida Engenheiro Soares de Camargo, 629 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>133</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>(11) 2155-8800</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr"/>
+          <t>(11) 99110-4782</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>(11) 2744-0100</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="38" customHeight="1">
       <c r="A26" s="3" t="n">
@@ -1194,27 +1198,27 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-169m2-venda-RS795000-id-2567773185/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-135m2-venda-RS850000-id-2846899624/</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Araruama, 158 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>135</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>(11) 96593-5749</t>
+          <t>(11) 99110-4782</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>(11) 2682-2320</t>
+          <t>(11) 2744-0100</t>
         </is>
       </c>
     </row>
@@ -1224,25 +1228,29 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-190m2-venda-RS890000-id-2869660708/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-139m2-venda-RS859000-id-2886562580/</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Rua Mazagão, 65 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Clevelândia, 280 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>139</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>(11) 2155-8801</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr"/>
+          <t>(11) 99110-4782</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>(11) 2744-0100</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="38" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -1250,25 +1258,29 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-226m2-venda-RS790000-id-2795163419/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-142m2-venda-RS799000-id-2846900138/</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Rua Marialva, 294 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Vitória da Conquista, 174 A - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>142</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>(11) 2385-7633</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
+          <t>(11) 99110-4782</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>(11) 2744-0100</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="38" customHeight="1">
       <c r="A29" s="8" t="n">
@@ -1276,29 +1288,25 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-227m2-venda-RS641000-id-2833843713/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-226m2-venda-RS790000-id-2795163419/</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Rua Mazagão, 322 - Cidade Patriarca, São Paulo - SP</t>
+          <t>Rua Marialva, 294 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>226</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>(11) 97395-3363</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>(11) 3565-3530</t>
-        </is>
-      </c>
+          <t>(11) 2385-7633</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="38" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -1306,27 +1314,27 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-263m2-venda-RS990000-id-2804358420/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-227m2-venda-RS641000-id-2833843713/</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Mazagão, 322 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>227</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>(11) 94084-8316</t>
+          <t>(11) 97395-3363</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>(11) 2958-8884</t>
+          <t>(11) 3565-3530</t>
         </is>
       </c>
     </row>
@@ -1336,27 +1344,27 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-287m2-venda-RS1150000-id-2840293965/</t>
+          <t>https://www.vivareal.com.br/imovel/sobrado-3-quartos-cidade-patriarca-zona-leste-sao-paulo-com-garagem-83m2-venda-RS400000-id-2746858359/</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>CEP 08079-354</t>
+          <t>Rua Quintiliano Moreira César, 104 - Cidade Patriarca, São Paulo - SP</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>(11) 96272-6666</t>
+          <t>(11) 96593-5749</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>(11) 2287-6666</t>
+          <t>(11) 2682-2320</t>
         </is>
       </c>
     </row>

</xml_diff>